<commit_message>
save 06 03 2026
</commit_message>
<xml_diff>
--- a/4 четверть_1_HTML_CSS_свойства 3 - респонсив, адаптив, ppi, img.xlsx
+++ b/4 четверть_1_HTML_CSS_свойства 3 - респонсив, адаптив, ppi, img.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Machenike\Desktop\Homework_repo\GB_Developer_Workbook\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA640E51-2533-4D8E-A8D3-F655FF5C2A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817C3149-8B8C-4AD8-8680-09B930824692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" tabRatio="825" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12840" yWindow="-18930" windowWidth="23010" windowHeight="12210" tabRatio="825" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="@media респонсив, адаптив" sheetId="38" r:id="rId1"/>
@@ -22,12 +22,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="158">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -4955,12 +4958,50 @@
       <t>- это размер экрана любого устройства, переведенный к ppi desktop (ppi desktop = 150). Полученный размер используется разработчиком в качестве размера экрана выбранного устройства (в данном случае выше - мобильного), чтобы понимать размер экрана и изображения, которые будут рзмещены на нем (должны быть не более полученного значения). А далее необходимо установить (либо через backgroud, либо через &lt;picture&gt;) медиа-запрос, который определит dpi конкретного устройства, определит размер экрана по формуле выше и подберет соответствующее изображение x1,x2,x3.. для отображения.</t>
     </r>
   </si>
+  <si>
+    <t>НОВОЕ!</t>
+  </si>
+  <si>
+    <t>Новый синтаксис медиазапросов Media Queries Range
+Если кто-то вдруг пропустил, то теперь медиазапросы можно писать проще и понятнее.
+Раньше нужно было делать так:</t>
+  </si>
+  <si>
+    <t>@media (max-width: 1000px) {
+    /* ... */
+}
+@media (min-width: 1000px) and (max-width: 1400px) {
+    /* ... */
+}</t>
+  </si>
+  <si>
+    <t>Раньше</t>
+  </si>
+  <si>
+    <t>Теперь</t>
+  </si>
+  <si>
+    <t>@media (width &lt;= 1000px) {
+    /* ... */
+}
+@media (1000px &lt;= width &lt;= 1400px) {
+    /* ... */
+}</t>
+  </si>
+  <si>
+    <t>В целом доступны такие операторы сравнения:
+■ &lt; — меньше;
+■ &gt; — больше;
+■ = — равно;
+■ &lt;= — меньше или равно;
+■ &gt;= — больше или равно.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5181,8 +5222,17 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5225,6 +5275,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -5239,7 +5295,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -5359,10 +5415,16 @@
     <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5525,9 +5587,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2119753</xdr:colOff>
+      <xdr:colOff>2115943</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>868670</xdr:rowOff>
+      <xdr:rowOff>861050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5569,9 +5631,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1837765</xdr:colOff>
+      <xdr:colOff>1845385</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>1046219</xdr:rowOff>
+      <xdr:rowOff>1050029</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5596,6 +5658,50 @@
         <a:xfrm>
           <a:off x="3045013" y="37803044"/>
           <a:ext cx="1307352" cy="991310"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>410808</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>50391</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2292016</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>1234082</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D61720B-F337-474A-8039-A146D4D3633B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11224484" y="15380038"/>
+          <a:ext cx="1881208" cy="1183691"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5875,38 +5981,38 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V69"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.1796875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.26953125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.08984375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.90625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.90625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6328125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.90625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.81640625" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.81640625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.7265625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.90625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.1796875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.7265625" style="8"/>
-    <col min="21" max="21" width="67.7265625" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.36328125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.36328125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6328125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.453125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.26953125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
         <v>1</v>
       </c>
@@ -5914,7 +6020,7 @@
       <c r="C1" s="39"/>
       <c r="D1" s="39"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -5933,7 +6039,7 @@
       <c r="S2" s="5"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -5942,7 +6048,7 @@
       <c r="U3" s="1"/>
       <c r="V3" s="2"/>
     </row>
-    <row r="4" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>71</v>
       </c>
@@ -5953,7 +6059,7 @@
       <c r="U4" s="1"/>
       <c r="V4" s="2"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>47</v>
       </c>
@@ -5962,7 +6068,7 @@
       <c r="U5" s="1"/>
       <c r="V5" s="2"/>
     </row>
-    <row r="6" spans="1:22" ht="116" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>48</v>
       </c>
@@ -5979,7 +6085,7 @@
       <c r="U6" s="1"/>
       <c r="V6" s="2"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
@@ -5994,7 +6100,7 @@
       <c r="U7" s="1"/>
       <c r="V7" s="2"/>
     </row>
-    <row r="8" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22"/>
       <c r="C8" s="22" t="s">
         <v>54</v>
@@ -6003,7 +6109,7 @@
       <c r="U8" s="1"/>
       <c r="V8" s="2"/>
     </row>
-    <row r="9" spans="1:22" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" ht="216" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>55</v>
       </c>
@@ -6020,7 +6126,7 @@
       <c r="U9" s="1"/>
       <c r="V9" s="2"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="23" t="s">
         <v>59</v>
       </c>
@@ -6035,7 +6141,7 @@
       <c r="U10" s="1"/>
       <c r="V10" s="2"/>
     </row>
-    <row r="11" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A11" s="22"/>
       <c r="B11" s="12" t="s">
         <v>61</v>
@@ -6048,7 +6154,7 @@
       <c r="U11" s="1"/>
       <c r="V11" s="2"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
         <v>63</v>
       </c>
@@ -6059,7 +6165,7 @@
       <c r="U12" s="1"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A13" s="22"/>
       <c r="B13" s="12" t="s">
         <v>64</v>
@@ -6072,7 +6178,7 @@
       <c r="U13" s="1"/>
       <c r="V13" s="2"/>
     </row>
-    <row r="14" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="23" t="s">
         <v>66</v>
       </c>
@@ -6089,7 +6195,7 @@
       <c r="U14" s="1"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="A15" s="22"/>
       <c r="B15" s="12" t="s">
         <v>61</v>
@@ -6104,7 +6210,7 @@
       <c r="U15" s="1"/>
       <c r="V15" s="2"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>72</v>
       </c>
@@ -6112,7 +6218,7 @@
       <c r="U16" s="1"/>
       <c r="V16" s="2"/>
     </row>
-    <row r="17" spans="1:22" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B17" s="15" t="s">
         <v>30</v>
       </c>
@@ -6123,7 +6229,7 @@
       <c r="U17" s="1"/>
       <c r="V17" s="2"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" s="36" t="s">
         <v>149</v>
       </c>
@@ -6132,7 +6238,7 @@
       <c r="U18" s="1"/>
       <c r="V18" s="2"/>
     </row>
-    <row r="19" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="B19" s="2" t="s">
         <v>142</v>
       </c>
@@ -6143,7 +6249,7 @@
       <c r="U19" s="1"/>
       <c r="V19" s="2"/>
     </row>
-    <row r="20" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="38" t="s">
         <v>144</v>
       </c>
@@ -6152,7 +6258,7 @@
       <c r="U20" s="1"/>
       <c r="V20" s="2"/>
     </row>
-    <row r="21" spans="1:22" ht="174" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" ht="172.8" x14ac:dyDescent="0.3">
       <c r="C21" s="37" t="s">
         <v>145</v>
       </c>
@@ -6160,7 +6266,7 @@
       <c r="U21" s="1"/>
       <c r="V21" s="2"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="38" t="s">
         <v>146</v>
       </c>
@@ -6169,7 +6275,7 @@
       <c r="U22" s="1"/>
       <c r="V22" s="2"/>
     </row>
-    <row r="23" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>147</v>
       </c>
@@ -6180,14 +6286,14 @@
       <c r="U23" s="1"/>
       <c r="V23" s="2"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B24" s="15"/>
       <c r="C24" s="25"/>
       <c r="P24" s="1"/>
       <c r="U24" s="1"/>
       <c r="V24" s="2"/>
     </row>
-    <row r="25" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
         <v>46</v>
       </c>
@@ -6212,28 +6318,28 @@
       <c r="U25" s="2"/>
       <c r="V25" s="1"/>
     </row>
-    <row r="26" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C26" s="13" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="C27" s="13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="C29" s="16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B30" s="2" t="s">
         <v>14</v>
       </c>
@@ -6241,7 +6347,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B31" s="2" t="s">
         <v>14</v>
       </c>
@@ -6249,7 +6355,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B32" s="2" t="s">
         <v>13</v>
       </c>
@@ -6257,7 +6363,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B33" s="2" t="s">
         <v>13</v>
       </c>
@@ -6265,7 +6371,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B34" s="2" t="s">
         <v>12</v>
       </c>
@@ -6273,7 +6379,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B35" s="2" t="s">
         <v>11</v>
       </c>
@@ -6281,43 +6387,43 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="C37" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C38" s="13"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C39" s="16" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C40" s="16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C41" s="16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="14" t="s">
         <v>19</v>
@@ -6326,7 +6432,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="174" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" ht="172.8" x14ac:dyDescent="0.3">
       <c r="B44" s="2" t="s">
         <v>25</v>
       </c>
@@ -6334,7 +6440,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="145" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="B45" s="2" t="s">
         <v>21</v>
       </c>
@@ -6342,7 +6448,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B46" s="14" t="s">
         <v>20</v>
       </c>
@@ -6350,7 +6456,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="116" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B47" s="14" t="s">
         <v>26</v>
       </c>
@@ -6358,7 +6464,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A48" s="17" t="s">
         <v>38</v>
       </c>
@@ -6366,7 +6472,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A49" s="18" t="s">
         <v>43</v>
       </c>
@@ -6377,7 +6483,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B50" s="2" t="s">
         <v>39</v>
       </c>
@@ -6385,7 +6491,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
         <v>37</v>
       </c>
@@ -6393,7 +6499,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="174" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
       <c r="B52" s="2" t="s">
         <v>41</v>
       </c>
@@ -6401,7 +6507,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="145" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="B53" s="2" t="s">
         <v>42</v>
       </c>
@@ -6409,33 +6515,33 @@
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="C62" s="30"/>
       <c r="D62" s="30"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
       <c r="C63" s="30"/>
       <c r="D63" s="30"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D64" s="30"/>
     </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D65" s="30"/>
     </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C66" s="29"/>
     </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C67" s="29"/>
     </row>
-    <row r="68" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C68" s="29"/>
       <c r="D68" s="29"/>
     </row>
-    <row r="69" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B69" s="30"/>
       <c r="C69" s="29"/>
       <c r="D69" s="2"/>
@@ -6456,39 +6562,39 @@
     <tabColor theme="7" tint="0.39997558519241921"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V53"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:V62"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.1796875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.26953125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.08984375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.90625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.90625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6328125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.90625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.81640625" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.81640625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.7265625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.90625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.1796875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.7265625" style="8"/>
-    <col min="21" max="21" width="67.7265625" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.36328125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.36328125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6328125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.453125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.26953125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
         <v>1</v>
       </c>
@@ -6496,7 +6602,7 @@
       <c r="C1" s="39"/>
       <c r="D1" s="39"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -6515,7 +6621,7 @@
       <c r="S2" s="5"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>135</v>
       </c>
@@ -6538,7 +6644,7 @@
       <c r="U3" s="2"/>
       <c r="V3" s="1"/>
     </row>
-    <row r="4" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="28" t="s">
         <v>75</v>
       </c>
@@ -6561,7 +6667,7 @@
       <c r="U4" s="2"/>
       <c r="V4" s="1"/>
     </row>
-    <row r="5" spans="1:22" s="7" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" s="7" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>77</v>
       </c>
@@ -6590,7 +6696,7 @@
       <c r="U5" s="2"/>
       <c r="V5" s="1"/>
     </row>
-    <row r="6" spans="1:22" s="7" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" s="7" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>76</v>
       </c>
@@ -6617,7 +6723,7 @@
       <c r="U6" s="2"/>
       <c r="V6" s="1"/>
     </row>
-    <row r="7" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="20" t="s">
         <v>85</v>
       </c>
@@ -6640,7 +6746,7 @@
       <c r="U7" s="2"/>
       <c r="V7" s="1"/>
     </row>
-    <row r="8" spans="1:22" s="7" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" s="7" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="30" t="s">
@@ -6663,7 +6769,7 @@
       <c r="U8" s="2"/>
       <c r="V8" s="1"/>
     </row>
-    <row r="9" spans="1:22" s="7" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" s="7" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="12"/>
       <c r="C9" s="30" t="s">
@@ -6686,7 +6792,7 @@
       <c r="U9" s="2"/>
       <c r="V9" s="1"/>
     </row>
-    <row r="10" spans="1:22" s="7" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" s="7" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="30" t="s">
@@ -6709,7 +6815,7 @@
       <c r="U10" s="2"/>
       <c r="V10" s="1"/>
     </row>
-    <row r="11" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
         <v>97</v>
       </c>
@@ -6734,7 +6840,7 @@
       <c r="U11" s="2"/>
       <c r="V11" s="1"/>
     </row>
-    <row r="12" spans="1:22" s="7" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" s="7" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="30" t="s">
@@ -6759,7 +6865,7 @@
       <c r="U12" s="2"/>
       <c r="V12" s="1"/>
     </row>
-    <row r="13" spans="1:22" s="7" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" s="7" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>86</v>
       </c>
@@ -6784,7 +6890,7 @@
       <c r="U13" s="2"/>
       <c r="V13" s="1"/>
     </row>
-    <row r="14" spans="1:22" s="7" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" s="7" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="30" t="s">
@@ -6807,7 +6913,7 @@
       <c r="U14" s="2"/>
       <c r="V14" s="1"/>
     </row>
-    <row r="15" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="20" t="s">
         <v>98</v>
       </c>
@@ -6836,7 +6942,7 @@
       <c r="U15" s="2"/>
       <c r="V15" s="1"/>
     </row>
-    <row r="16" spans="1:22" s="7" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" s="7" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>99</v>
       </c>
@@ -6865,7 +6971,7 @@
       <c r="U16" s="2"/>
       <c r="V16" s="1"/>
     </row>
-    <row r="17" spans="1:22" s="7" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" s="7" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="30" t="s">
         <v>120</v>
@@ -6892,7 +6998,7 @@
       <c r="U17" s="2"/>
       <c r="V17" s="1"/>
     </row>
-    <row r="18" spans="1:22" s="7" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" s="7" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>100</v>
       </c>
@@ -6921,15 +7027,15 @@
       <c r="U18" s="2"/>
       <c r="V18" s="1"/>
     </row>
-    <row r="19" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="B19" s="40" t="s">
-        <v>133</v>
-      </c>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
+      <c r="B19" s="42" t="s">
+        <v>151</v>
+      </c>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
       <c r="F19" s="1"/>
       <c r="G19" s="2"/>
       <c r="H19" s="1"/>
@@ -6946,14 +7052,16 @@
       <c r="U19" s="2"/>
       <c r="V19" s="1"/>
     </row>
-    <row r="20" spans="1:22" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C20" s="4"/>
+    <row r="20" spans="1:22" s="7" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B20" s="41" t="s">
+        <v>153</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>152</v>
+      </c>
       <c r="D20" s="30"/>
       <c r="F20" s="1"/>
       <c r="G20" s="2"/>
@@ -6971,15 +7079,17 @@
       <c r="U20" s="2"/>
       <c r="V20" s="1"/>
     </row>
-    <row r="21" spans="1:22" s="7" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="1"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="D21" s="30" t="s">
-        <v>121</v>
-      </c>
+    <row r="21" spans="1:22" s="7" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>156</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="D21" s="30"/>
       <c r="F21" s="1"/>
       <c r="G21" s="2"/>
       <c r="H21" s="1"/>
@@ -6996,16 +7106,10 @@
       <c r="U21" s="2"/>
       <c r="V21" s="1"/>
     </row>
-    <row r="22" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C22" s="35" t="s">
-        <v>140</v>
-      </c>
+    <row r="22" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
       <c r="D22" s="30"/>
       <c r="F22" s="1"/>
       <c r="G22" s="2"/>
@@ -7023,12 +7127,10 @@
       <c r="U22" s="2"/>
       <c r="V22" s="1"/>
     </row>
-    <row r="23" spans="1:22" s="7" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="1"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="35" t="s">
-        <v>141</v>
-      </c>
+    <row r="23" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="2"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
       <c r="D23" s="30"/>
       <c r="F23" s="1"/>
       <c r="G23" s="2"/>
@@ -7046,14 +7148,10 @@
       <c r="U23" s="2"/>
       <c r="V23" s="1"/>
     </row>
-    <row r="24" spans="1:22" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C24" s="4"/>
+    <row r="24" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
       <c r="D24" s="30"/>
       <c r="F24" s="1"/>
       <c r="G24" s="2"/>
@@ -7071,14 +7169,10 @@
       <c r="U24" s="2"/>
       <c r="V24" s="1"/>
     </row>
-    <row r="25" spans="1:22" s="7" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="A25" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="27" t="s">
-        <v>73</v>
-      </c>
+    <row r="25" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
       <c r="D25" s="30"/>
       <c r="F25" s="1"/>
       <c r="G25" s="2"/>
@@ -7096,16 +7190,10 @@
       <c r="U25" s="2"/>
       <c r="V25" s="1"/>
     </row>
-    <row r="26" spans="1:22" s="7" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" s="30" t="s">
-        <v>132</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>74</v>
-      </c>
+    <row r="26" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="2"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="30"/>
       <c r="D26" s="30"/>
       <c r="F26" s="1"/>
       <c r="G26" s="2"/>
@@ -7123,14 +7211,10 @@
       <c r="U26" s="2"/>
       <c r="V26" s="1"/>
     </row>
-    <row r="27" spans="1:22" s="7" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="29" t="s">
-        <v>80</v>
-      </c>
+    <row r="27" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="2"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="30"/>
       <c r="D27" s="30"/>
       <c r="F27" s="1"/>
       <c r="G27" s="2"/>
@@ -7148,13 +7232,15 @@
       <c r="U27" s="2"/>
       <c r="V27" s="1"/>
     </row>
-    <row r="28" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
+    <row r="28" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="40" t="s">
+        <v>133</v>
+      </c>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
       <c r="F28" s="1"/>
       <c r="G28" s="2"/>
       <c r="H28" s="1"/>
@@ -7171,12 +7257,14 @@
       <c r="U28" s="2"/>
       <c r="V28" s="1"/>
     </row>
-    <row r="29" spans="1:22" s="7" customFormat="1" ht="87" x14ac:dyDescent="0.35">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="30" t="s">
-        <v>114</v>
-      </c>
+    <row r="29" spans="1:22" s="7" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C29" s="4"/>
       <c r="D29" s="30"/>
       <c r="F29" s="1"/>
       <c r="G29" s="2"/>
@@ -7194,15 +7282,15 @@
       <c r="U29" s="2"/>
       <c r="V29" s="1"/>
     </row>
-    <row r="30" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="C30" s="32"/>
-      <c r="D30" s="33"/>
+    <row r="30" spans="1:22" s="7" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A30" s="1"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>121</v>
+      </c>
       <c r="F30" s="1"/>
       <c r="G30" s="2"/>
       <c r="H30" s="1"/>
@@ -7219,11 +7307,15 @@
       <c r="U30" s="2"/>
       <c r="V30" s="1"/>
     </row>
-    <row r="31" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2" t="s">
-        <v>105</v>
+    <row r="31" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C31" s="35" t="s">
+        <v>140</v>
       </c>
       <c r="D31" s="30"/>
       <c r="F31" s="1"/>
@@ -7242,17 +7334,13 @@
       <c r="U31" s="2"/>
       <c r="V31" s="1"/>
     </row>
-    <row r="32" spans="1:22" s="7" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="30"/>
-      <c r="B32" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D32" s="30" t="s">
-        <v>117</v>
-      </c>
+    <row r="32" spans="1:22" s="7" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="A32" s="1"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="35" t="s">
+        <v>141</v>
+      </c>
+      <c r="D32" s="30"/>
       <c r="F32" s="1"/>
       <c r="G32" s="2"/>
       <c r="H32" s="1"/>
@@ -7269,16 +7357,14 @@
       <c r="U32" s="2"/>
       <c r="V32" s="1"/>
     </row>
-    <row r="33" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="B33" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="C33" s="20" t="s">
-        <v>107</v>
-      </c>
+    <row r="33" spans="1:22" s="7" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C33" s="4"/>
       <c r="D33" s="30"/>
       <c r="F33" s="1"/>
       <c r="G33" s="2"/>
@@ -7296,17 +7382,15 @@
       <c r="U33" s="2"/>
       <c r="V33" s="1"/>
     </row>
-    <row r="34" spans="1:22" s="7" customFormat="1" ht="203" x14ac:dyDescent="0.35">
-      <c r="A34" s="1"/>
-      <c r="B34" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D34" s="30" t="s">
-        <v>113</v>
-      </c>
+    <row r="34" spans="1:22" s="7" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="B34" s="2"/>
+      <c r="C34" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="30"/>
       <c r="F34" s="1"/>
       <c r="G34" s="2"/>
       <c r="H34" s="1"/>
@@ -7323,15 +7407,17 @@
       <c r="U34" s="2"/>
       <c r="V34" s="1"/>
     </row>
-    <row r="35" spans="1:22" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="C35" s="32"/>
-      <c r="D35" s="33"/>
+    <row r="35" spans="1:22" s="7" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" s="30"/>
       <c r="F35" s="1"/>
       <c r="G35" s="2"/>
       <c r="H35" s="1"/>
@@ -7348,13 +7434,13 @@
       <c r="U35" s="2"/>
       <c r="V35" s="1"/>
     </row>
-    <row r="36" spans="1:22" s="7" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" s="7" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="B36" s="2"/>
-      <c r="C36" s="30" t="s">
-        <v>119</v>
+      <c r="C36" s="29" t="s">
+        <v>80</v>
       </c>
       <c r="D36" s="30"/>
       <c r="F36" s="1"/>
@@ -7373,179 +7459,405 @@
       <c r="U36" s="2"/>
       <c r="V36" s="1"/>
     </row>
-    <row r="46" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-      <c r="K46" s="1"/>
-      <c r="L46" s="1"/>
-      <c r="M46" s="1"/>
-      <c r="N46" s="1"/>
-      <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
-      <c r="R46" s="2"/>
-      <c r="S46" s="1"/>
-      <c r="T46" s="8"/>
-      <c r="U46" s="2"/>
-      <c r="V46" s="1"/>
-    </row>
-    <row r="47" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="F47" s="1"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-      <c r="K47" s="1"/>
-      <c r="L47" s="1"/>
-      <c r="M47" s="1"/>
-      <c r="N47" s="1"/>
-      <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
-      <c r="R47" s="2"/>
-      <c r="S47" s="1"/>
-      <c r="T47" s="8"/>
-      <c r="U47" s="2"/>
-      <c r="V47" s="1"/>
-    </row>
-    <row r="48" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="1"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="30"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="2"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="K48" s="1"/>
-      <c r="L48" s="1"/>
-      <c r="M48" s="1"/>
-      <c r="N48" s="1"/>
-      <c r="P48" s="2"/>
-      <c r="Q48" s="2"/>
-      <c r="R48" s="2"/>
-      <c r="S48" s="1"/>
-      <c r="T48" s="8"/>
-      <c r="U48" s="2"/>
-      <c r="V48" s="1"/>
-    </row>
-    <row r="49" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="1"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="30"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="2"/>
-      <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-      <c r="K49" s="1"/>
-      <c r="L49" s="1"/>
-      <c r="M49" s="1"/>
-      <c r="N49" s="1"/>
-      <c r="P49" s="2"/>
-      <c r="Q49" s="2"/>
-      <c r="R49" s="2"/>
-      <c r="S49" s="1"/>
-      <c r="T49" s="8"/>
-      <c r="U49" s="2"/>
-      <c r="V49" s="1"/>
-    </row>
-    <row r="50" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="1"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-      <c r="K50" s="1"/>
-      <c r="L50" s="1"/>
-      <c r="M50" s="1"/>
-      <c r="N50" s="1"/>
-      <c r="P50" s="2"/>
-      <c r="Q50" s="2"/>
-      <c r="R50" s="2"/>
-      <c r="S50" s="1"/>
-      <c r="T50" s="8"/>
-      <c r="U50" s="2"/>
-      <c r="V50" s="1"/>
-    </row>
-    <row r="51" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="1"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="1"/>
-      <c r="F51" s="1"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-      <c r="K51" s="1"/>
-      <c r="L51" s="1"/>
-      <c r="M51" s="1"/>
-      <c r="N51" s="1"/>
-      <c r="P51" s="2"/>
-      <c r="Q51" s="2"/>
-      <c r="R51" s="2"/>
-      <c r="S51" s="1"/>
-      <c r="T51" s="8"/>
-      <c r="U51" s="2"/>
-      <c r="V51" s="1"/>
-    </row>
-    <row r="52" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="1"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="29"/>
-      <c r="D52" s="29"/>
-      <c r="F52" s="1"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="1"/>
-      <c r="I52" s="1"/>
-      <c r="K52" s="1"/>
-      <c r="L52" s="1"/>
-      <c r="M52" s="1"/>
-      <c r="N52" s="1"/>
-      <c r="P52" s="2"/>
-      <c r="Q52" s="2"/>
-      <c r="R52" s="2"/>
-      <c r="S52" s="1"/>
-      <c r="T52" s="8"/>
-      <c r="U52" s="2"/>
-      <c r="V52" s="1"/>
-    </row>
-    <row r="53" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="1"/>
-      <c r="B53" s="30"/>
-      <c r="C53" s="29"/>
-      <c r="D53" s="2"/>
-      <c r="F53" s="1"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="1"/>
-      <c r="I53" s="1"/>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-      <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-      <c r="P53" s="2"/>
-      <c r="Q53" s="2"/>
-      <c r="R53" s="2"/>
-      <c r="S53" s="1"/>
-      <c r="T53" s="8"/>
-      <c r="U53" s="2"/>
-      <c r="V53" s="1"/>
+    <row r="37" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" s="19"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="P37" s="2"/>
+      <c r="Q37" s="2"/>
+      <c r="R37" s="2"/>
+      <c r="S37" s="1"/>
+      <c r="T37" s="8"/>
+      <c r="U37" s="2"/>
+      <c r="V37" s="1"/>
+    </row>
+    <row r="38" spans="1:22" s="7" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="D38" s="30"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="P38" s="2"/>
+      <c r="Q38" s="2"/>
+      <c r="R38" s="2"/>
+      <c r="S38" s="1"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="2"/>
+      <c r="V38" s="1"/>
+    </row>
+    <row r="39" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C39" s="32"/>
+      <c r="D39" s="33"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="P39" s="2"/>
+      <c r="Q39" s="2"/>
+      <c r="R39" s="2"/>
+      <c r="S39" s="1"/>
+      <c r="T39" s="8"/>
+      <c r="U39" s="2"/>
+      <c r="V39" s="1"/>
+    </row>
+    <row r="40" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" s="30"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
+      <c r="P40" s="2"/>
+      <c r="Q40" s="2"/>
+      <c r="R40" s="2"/>
+      <c r="S40" s="1"/>
+      <c r="T40" s="8"/>
+      <c r="U40" s="2"/>
+      <c r="V40" s="1"/>
+    </row>
+    <row r="41" spans="1:22" s="7" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="30"/>
+      <c r="B41" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="F41" s="1"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="K41" s="1"/>
+      <c r="L41" s="1"/>
+      <c r="M41" s="1"/>
+      <c r="N41" s="1"/>
+      <c r="P41" s="2"/>
+      <c r="Q41" s="2"/>
+      <c r="R41" s="2"/>
+      <c r="S41" s="1"/>
+      <c r="T41" s="8"/>
+      <c r="U41" s="2"/>
+      <c r="V41" s="1"/>
+    </row>
+    <row r="42" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A42" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="C42" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="D42" s="30"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+      <c r="K42" s="1"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
+      <c r="P42" s="2"/>
+      <c r="Q42" s="2"/>
+      <c r="R42" s="2"/>
+      <c r="S42" s="1"/>
+      <c r="T42" s="8"/>
+      <c r="U42" s="2"/>
+      <c r="V42" s="1"/>
+    </row>
+    <row r="43" spans="1:22" s="7" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="1"/>
+      <c r="B43" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D43" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="F43" s="1"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1"/>
+      <c r="K43" s="1"/>
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
+      <c r="P43" s="2"/>
+      <c r="Q43" s="2"/>
+      <c r="R43" s="2"/>
+      <c r="S43" s="1"/>
+      <c r="T43" s="8"/>
+      <c r="U43" s="2"/>
+      <c r="V43" s="1"/>
+    </row>
+    <row r="44" spans="1:22" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A44" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="C44" s="32"/>
+      <c r="D44" s="33"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="P44" s="2"/>
+      <c r="Q44" s="2"/>
+      <c r="R44" s="2"/>
+      <c r="S44" s="1"/>
+      <c r="T44" s="8"/>
+      <c r="U44" s="2"/>
+      <c r="V44" s="1"/>
+    </row>
+    <row r="45" spans="1:22" s="7" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="D45" s="30"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+      <c r="K45" s="1"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
+      <c r="P45" s="2"/>
+      <c r="Q45" s="2"/>
+      <c r="R45" s="2"/>
+      <c r="S45" s="1"/>
+      <c r="T45" s="8"/>
+      <c r="U45" s="2"/>
+      <c r="V45" s="1"/>
+    </row>
+    <row r="55" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="30"/>
+      <c r="D55" s="30"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1"/>
+      <c r="K55" s="1"/>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+      <c r="N55" s="1"/>
+      <c r="P55" s="2"/>
+      <c r="Q55" s="2"/>
+      <c r="R55" s="2"/>
+      <c r="S55" s="1"/>
+      <c r="T55" s="8"/>
+      <c r="U55" s="2"/>
+      <c r="V55" s="1"/>
+    </row>
+    <row r="56" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="30"/>
+      <c r="D56" s="30"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
+      <c r="K56" s="1"/>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+      <c r="N56" s="1"/>
+      <c r="P56" s="2"/>
+      <c r="Q56" s="2"/>
+      <c r="R56" s="2"/>
+      <c r="S56" s="1"/>
+      <c r="T56" s="8"/>
+      <c r="U56" s="2"/>
+      <c r="V56" s="1"/>
+    </row>
+    <row r="57" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="1"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="30"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="1"/>
+      <c r="K57" s="1"/>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+      <c r="N57" s="1"/>
+      <c r="P57" s="2"/>
+      <c r="Q57" s="2"/>
+      <c r="R57" s="2"/>
+      <c r="S57" s="1"/>
+      <c r="T57" s="8"/>
+      <c r="U57" s="2"/>
+      <c r="V57" s="1"/>
+    </row>
+    <row r="58" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="1"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="30"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+      <c r="N58" s="1"/>
+      <c r="P58" s="2"/>
+      <c r="Q58" s="2"/>
+      <c r="R58" s="2"/>
+      <c r="S58" s="1"/>
+      <c r="T58" s="8"/>
+      <c r="U58" s="2"/>
+      <c r="V58" s="1"/>
+    </row>
+    <row r="59" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="1"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="1"/>
+      <c r="K59" s="1"/>
+      <c r="L59" s="1"/>
+      <c r="M59" s="1"/>
+      <c r="N59" s="1"/>
+      <c r="P59" s="2"/>
+      <c r="Q59" s="2"/>
+      <c r="R59" s="2"/>
+      <c r="S59" s="1"/>
+      <c r="T59" s="8"/>
+      <c r="U59" s="2"/>
+      <c r="V59" s="1"/>
+    </row>
+    <row r="60" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="1"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="29"/>
+      <c r="D60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
+      <c r="N60" s="1"/>
+      <c r="P60" s="2"/>
+      <c r="Q60" s="2"/>
+      <c r="R60" s="2"/>
+      <c r="S60" s="1"/>
+      <c r="T60" s="8"/>
+      <c r="U60" s="2"/>
+      <c r="V60" s="1"/>
+    </row>
+    <row r="61" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="1"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="29"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="1"/>
+      <c r="I61" s="1"/>
+      <c r="K61" s="1"/>
+      <c r="L61" s="1"/>
+      <c r="M61" s="1"/>
+      <c r="N61" s="1"/>
+      <c r="P61" s="2"/>
+      <c r="Q61" s="2"/>
+      <c r="R61" s="2"/>
+      <c r="S61" s="1"/>
+      <c r="T61" s="8"/>
+      <c r="U61" s="2"/>
+      <c r="V61" s="1"/>
+    </row>
+    <row r="62" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="1"/>
+      <c r="B62" s="30"/>
+      <c r="C62" s="29"/>
+      <c r="D62" s="2"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="2"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="1"/>
+      <c r="K62" s="1"/>
+      <c r="L62" s="1"/>
+      <c r="M62" s="1"/>
+      <c r="N62" s="1"/>
+      <c r="P62" s="2"/>
+      <c r="Q62" s="2"/>
+      <c r="R62" s="2"/>
+      <c r="S62" s="1"/>
+      <c r="T62" s="8"/>
+      <c r="U62" s="2"/>
+      <c r="V62" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B11:D11"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B11:D11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D5" r:id="rId1" location=":~:text=%D0%A7%D1%82%D0%BE%20%D1%82%D0%B0%D0%BA%D0%BE%D0%B5%20DPI%20%D0%B8%20PPI&amp;text=%D0%A7%D0%B5%D0%BC%20%D0%BC%D0%B5%D0%BD%D1%8C%D1%88%D0%B5%20DPI%2C%20%D1%82%D0%B5%D0%BC%20%D0%BC%D0%B5%D0%BD%D0%B5%D0%B5,%D1%81%D0%BF%D0%BE%D1%81%D0%BE%D0%B1%D0%B5%D0%BD%20%D0%BE%D1%82%D0%BE%D0%B1%D1%80%D0%B0%D0%B7%D0%B8%D1%82%D1%8C%20%D0%BD%D0%B0%201%20%D0%B4%D1%8E%D0%B9%D0%BC%D0%B5." xr:uid="{D74DE2CE-CDC1-4810-9B54-4C30C27A039C}"/>
@@ -7562,38 +7874,38 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.1796875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.26953125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.08984375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.90625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.90625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6328125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.90625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.81640625" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.81640625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.7265625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.90625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.1796875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.7265625" style="8"/>
-    <col min="21" max="21" width="67.7265625" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.36328125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.36328125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6328125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.453125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.26953125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
         <v>1</v>
       </c>
@@ -7601,7 +7913,7 @@
       <c r="C1" s="39"/>
       <c r="D1" s="39"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -7620,7 +7932,7 @@
       <c r="S2" s="5"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -7629,7 +7941,7 @@
       <c r="U3" s="1"/>
       <c r="V3" s="2"/>
     </row>
-    <row r="4" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
       <c r="B4" s="2"/>
       <c r="C4" s="4"/>

</xml_diff>